<commit_message>
Corrige validação do cronograma audiovisual
</commit_message>
<xml_diff>
--- a/outputs/aula-03/PA_A03_MODELO_CRONOGRAMA.xlsx
+++ b/outputs/aula-03/PA_A03_MODELO_CRONOGRAMA.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMECE_AQUI" sheetId="1" r:id="Rd8addf717aa54980"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_FLUXO" sheetId="2" r:id="R63b8c9b806f44735"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_GENEROS" sheetId="3" r:id="Rafff794bc71e4398"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_CRONOGRAMA" sheetId="4" r:id="R06f1e919fe984801"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_CONFERENCIA" sheetId="5" r:id="Rc3c78daa1cd84e52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMECE_AQUI" sheetId="1" r:id="Rf0ad490dcba04a41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_FLUXO" sheetId="2" r:id="R949f1dc3c7174f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_GENEROS" sheetId="3" r:id="R164fafa348d2491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_CRONOGRAMA" sheetId="4" r:id="Rd459dc4a45c64db3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_CONFERENCIA" sheetId="5" r:id="Rda47e45f220c4848"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -583,7 +583,7 @@
         <x:color rgb="FF171915"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEFF5C6"/>
         </x:patternFill>
       </x:fill>
@@ -594,7 +594,7 @@
         <x:color rgb="FF171915"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEFF5C6"/>
         </x:patternFill>
       </x:fill>
@@ -605,7 +605,7 @@
         <x:color rgb="FF171915"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEFF5C6"/>
         </x:patternFill>
       </x:fill>
@@ -616,7 +616,7 @@
         <x:color rgb="FF171915"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEFF5C6"/>
         </x:patternFill>
       </x:fill>
@@ -1829,7 +1829,7 @@
         <x:v>Tarefas</x:v>
       </x:c>
       <x:c r="K5" s="87" t="n">
-        <x:f>COUNTA(B9:B23)</x:f>
+        <x:f>COUNTIF(B9:B23,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1842,7 +1842,7 @@
         <x:v>Pré</x:v>
       </x:c>
       <x:c r="K6" s="87" t="n">
-        <x:f>COUNTIF(C9:C23,"PRÉ")</x:f>
+        <x:f>COUNTIFS(B9:B23,"&lt;&gt;",C9:C23,"PRÉ")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1851,7 +1851,7 @@
         <x:v>Produção</x:v>
       </x:c>
       <x:c r="K7" s="87" t="n">
-        <x:f>COUNTIF(C9:C23,"PRODUÇÃO")</x:f>
+        <x:f>COUNTIFS(B9:B23,"&lt;&gt;",C9:C23,"PRODUÇÃO")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1884,7 +1884,7 @@
         <x:v>Pós</x:v>
       </x:c>
       <x:c r="K8" s="87" t="n">
-        <x:f>COUNTIF(C9:C23,"PÓS")</x:f>
+        <x:f>COUNTIFS(B9:B23,"&lt;&gt;",C9:C23,"PÓS")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1903,7 +1903,7 @@
         <x:v>Responsáveis</x:v>
       </x:c>
       <x:c r="K9" s="87" t="n">
-        <x:f>COUNTA(D9:D23)</x:f>
+        <x:f>COUNTIFS(B9:B23,"&lt;&gt;",D9:D23,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1922,7 +1922,7 @@
         <x:v>Durações</x:v>
       </x:c>
       <x:c r="K10" s="87" t="n">
-        <x:f>COUNT(E9:E23)</x:f>
+        <x:f>COUNTIFS(B9:B23,"&lt;&gt;",E9:E23,"&gt;0")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1941,7 +1941,7 @@
         <x:v>Dependências</x:v>
       </x:c>
       <x:c r="K11" s="87" t="n">
-        <x:f>COUNTA(F9:F23)</x:f>
+        <x:f>COUNTIFS(B9:B23,"&lt;&gt;",F9:F23,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1960,7 +1960,7 @@
         <x:v>Evidências</x:v>
       </x:c>
       <x:c r="K12" s="87" t="n">
-        <x:f>COUNTA(G9:G23)</x:f>
+        <x:f>COUNTIFS(B9:B23,"&lt;&gt;",G9:G23,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2004,7 +2004,7 @@
       <x:c r="G15" s="36"/>
       <x:c r="H15" s="36"/>
       <x:c r="J15" s="96" t="str">
-        <x:f>IF(AND(K5&gt;=10,K6&gt;=4,K7&gt;=2,K8&gt;=4,K9&gt;=K5,K10&gt;=K5,K11&gt;=2,K12&gt;=K5),"CONCLUÍDO","PENDENTE")</x:f>
+        <x:f>IF(AND(K5&gt;=10,K6&gt;=4,K7&gt;=2,K8&gt;=4,K6+K7+K8=K5,K9=K5,K10=K5,K11&gt;=2,K12=K5),"CONCLUÍDO","PENDENTE")</x:f>
         <x:v>PENDENTE</x:v>
       </x:c>
       <x:c r="K15" s="97"/>

</xml_diff>